<commit_message>
add FDE stakeholder analysis artifacts
</commit_message>
<xml_diff>
--- a/src/FDE_GLS.xlsx
+++ b/src/FDE_GLS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dar/Documents/bsa-delivery-service-case-study/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94A14DB-4EE2-7045-8D5C-3E2F251E38BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221E8F99-7AF8-924C-A9E2-722B7E9B560C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{D2E70F53-19F9-BD47-AB3F-DBD826BEFA02}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="82">
   <si>
     <t>Код</t>
   </si>
@@ -204,6 +204,87 @@
   </si>
   <si>
     <t>FDE_GLS_013</t>
+  </si>
+  <si>
+    <t>FDE_GLS_014</t>
+  </si>
+  <si>
+    <t>Основатель</t>
+  </si>
+  <si>
+    <t>Это лицо, которое положило начало, создало, учредило или организовало что-либо</t>
+  </si>
+  <si>
+    <t>Зачинатель, основоположник</t>
+  </si>
+  <si>
+    <t>Грамота.ру</t>
+  </si>
+  <si>
+    <t>FDE_GLS_015</t>
+  </si>
+  <si>
+    <t>Индивидуальный клиент</t>
+  </si>
+  <si>
+    <t>Физическое лицо, которое приобретает товары или услуги для личного, семейного или домашнего использования, а не для перепродажи или бизнеса.</t>
+  </si>
+  <si>
+    <t>FDE_GLS_016</t>
+  </si>
+  <si>
+    <t>Магазин</t>
+  </si>
+  <si>
+    <t>Специально оборудованное стационарное здание или часть здания, предназначенное для продажи товаров.</t>
+  </si>
+  <si>
+    <t>Википедия</t>
+  </si>
+  <si>
+    <t>FDE_GLS_017</t>
+  </si>
+  <si>
+    <t>Предприятие питания</t>
+  </si>
+  <si>
+    <t>Объект хозяйственной деятельности, предназначенный для изготовления продукции общественного питания, создания условий для потребления и реализации продукции общественного питания и покупных товаров (в т.ч. пищевых продуктов промышленного изготовления), как на месте изготовления, так и вне его по заказам, а также для оказания разнообразных дополнительных услуг, в том числе по организации досуга потребителей.</t>
+  </si>
+  <si>
+    <t>Предприятие общественного питания</t>
+  </si>
+  <si>
+    <t>ГОСТ Р 50647-2010</t>
+  </si>
+  <si>
+    <t>FDE_GLS_018</t>
+  </si>
+  <si>
+    <t>Оператор</t>
+  </si>
+  <si>
+    <t>Юридическое или физическое лицо, которое организует и (или) осуществляет обработку персональных данных, а также определяет цели и содержание этой обработки.</t>
+  </si>
+  <si>
+    <t>№ 152-ФЗ «О персональных данных»</t>
+  </si>
+  <si>
+    <t>FDE_GLS_019</t>
+  </si>
+  <si>
+    <t>Администратор</t>
+  </si>
+  <si>
+    <t>Должностное лицо (специалист), управляющее в коллективе учреждения, организации, компании и так далее.</t>
+  </si>
+  <si>
+    <t>FDE_GLS_020</t>
+  </si>
+  <si>
+    <t>Бухгалтер</t>
+  </si>
+  <si>
+    <t>(нем. Buchhalter, Buch — книга, Halter — держатель/держатель книги) — специалист по бухгалтерскому учёту, работающий по системе учёта в соответствии с действующим законодательством.</t>
   </si>
 </sst>
 </file>
@@ -269,7 +350,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -331,11 +412,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -372,6 +464,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6EB0CF-0A09-5D48-83D2-35A5B3D8864C}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
@@ -1084,6 +1182,188 @@
         <v>12</v>
       </c>
     </row>
+    <row r="15" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+      <c r="A15" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F15" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+      <c r="A16" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A17" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G17" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="255" x14ac:dyDescent="0.2">
+      <c r="A18" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C18" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G18" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="102" x14ac:dyDescent="0.2">
+      <c r="A19" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G19" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+      <c r="A20" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G20" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+      <c r="A21" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="10">
+        <v>46236</v>
+      </c>
+      <c r="G21" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add FDE process and context artifacts
</commit_message>
<xml_diff>
--- a/src/FDE_GLS.xlsx
+++ b/src/FDE_GLS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dar/Documents/bsa-delivery-service-case-study/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{221E8F99-7AF8-924C-A9E2-722B7E9B560C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1160F9F-824F-4342-9914-9DFE56C4F1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{D2E70F53-19F9-BD47-AB3F-DBD826BEFA02}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="88">
   <si>
     <t>Код</t>
   </si>
@@ -285,6 +285,24 @@
   </si>
   <si>
     <t>(нем. Buchhalter, Buch — книга, Halter — держатель/держатель книги) — специалист по бухгалтерскому учёту, работающий по системе учёта в соответствии с действующим законодательством.</t>
+  </si>
+  <si>
+    <t>Требование</t>
+  </si>
+  <si>
+    <t>это пригодное для практического использования представление потребности или решения</t>
+  </si>
+  <si>
+    <t>Контекстная диаграмма</t>
+  </si>
+  <si>
+    <t>Она отображает, какие потоки информации или управляющие воздействия передаются извне внутрь системы, а какие из системы наружу, и кто их передает. Контекстная диаграмма не показывает, что делается внутри системы, только «черный ящик». А еще она помогает определить границы системы.</t>
+  </si>
+  <si>
+    <t>FDE_GLS_021</t>
+  </si>
+  <si>
+    <t>FDE_GLS_022</t>
   </si>
 </sst>
 </file>
@@ -805,7 +823,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC6EB0CF-0A09-5D48-83D2-35A5B3D8864C}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.1640625" customWidth="1"/>
@@ -1364,6 +1382,110 @@
         <v>12</v>
       </c>
     </row>
+    <row r="22" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A22" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="10">
+        <v>46237</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="160" x14ac:dyDescent="0.2">
+      <c r="A23" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="10">
+        <v>46237</v>
+      </c>
+      <c r="G23" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="48" x14ac:dyDescent="0.2">
+      <c r="A24" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F24" s="10">
+        <v>46237</v>
+      </c>
+      <c r="G24" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="160" x14ac:dyDescent="0.2">
+      <c r="A25" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F25" s="10">
+        <v>46237</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>